<commit_message>
Update Excel template with latest changes
</commit_message>
<xml_diff>
--- a/public/Electrical Consumption.xlsx
+++ b/public/Electrical Consumption.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Msi\Desktop\electrical-consumption-reporter\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F7EF638-F128-4A04-89D8-1AE516EFB8B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E51C77C-434B-40A8-ABD8-B7223149BEF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{3D1C84FC-D0D6-48B3-9275-4A3111EEBB06}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="54">
   <si>
     <t>Electrical Consumption Reporting</t>
   </si>
@@ -135,9 +135,6 @@
     <t>Total 6</t>
   </si>
   <si>
-    <t>Boiler</t>
-  </si>
-  <si>
     <t>PDB 3</t>
   </si>
   <si>
@@ -193,6 +190,15 @@
   </si>
   <si>
     <t>Chaudière</t>
+  </si>
+  <si>
+    <t>Zone 4</t>
+  </si>
+  <si>
+    <t>LYDEC Global</t>
+  </si>
+  <si>
+    <t>MT Room</t>
   </si>
 </sst>
 </file>
@@ -844,7 +850,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B3:H42"/>
+  <dimension ref="B3:H44"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="1"/>
@@ -987,7 +993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="3:8" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:6" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C17" s="11"/>
       <c r="D17" s="3" t="s">
         <v>19</v>
@@ -997,7 +1003,7 @@
       </c>
       <c r="F17" s="2"/>
     </row>
-    <row r="18" spans="3:8" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="3:6" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C18" s="12" t="s">
         <v>21</v>
       </c>
@@ -1008,7 +1014,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="3:8" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:6" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D19" s="17" t="s">
         <v>25</v>
       </c>
@@ -1017,14 +1023,14 @@
       </c>
       <c r="F19" s="2"/>
     </row>
-    <row r="20" spans="3:8" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:6" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D20" s="17"/>
       <c r="E20" s="5" t="s">
         <v>23</v>
       </c>
       <c r="F20" s="2"/>
     </row>
-    <row r="21" spans="3:8" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:6" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D21" s="17"/>
       <c r="E21" s="5" t="s">
         <v>7</v>
@@ -1034,7 +1040,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="3:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="3:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D22" s="17"/>
       <c r="E22" s="5" t="s">
         <v>8</v>
@@ -1044,7 +1050,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="3:8" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="3:6" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C23" s="12" t="s">
         <v>24</v>
       </c>
@@ -1055,7 +1061,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="3:8" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="3:6" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D24" s="4" t="s">
         <v>26</v>
       </c>
@@ -1064,7 +1070,7 @@
       </c>
       <c r="F24" s="2"/>
     </row>
-    <row r="25" spans="3:8" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="3:6" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C25" s="12" t="s">
         <v>28</v>
       </c>
@@ -1075,7 +1081,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="3:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="3:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D26" s="4" t="s">
         <v>29</v>
       </c>
@@ -1084,7 +1090,7 @@
       </c>
       <c r="F26" s="7"/>
     </row>
-    <row r="27" spans="3:8" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="3:6" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C27" s="12" t="s">
         <v>31</v>
       </c>
@@ -1095,158 +1101,171 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="3:8" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D28" s="4" t="s">
+    <row r="28" spans="3:6" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D28" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="F28" s="2"/>
+    </row>
+    <row r="29" spans="3:6" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D29" s="17"/>
+      <c r="E29" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="E28" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="F28" s="7"/>
-      <c r="G28" s="7" t="s">
+      <c r="F29" s="2"/>
+    </row>
+    <row r="30" spans="3:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C30" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="H28" s="7"/>
-    </row>
-    <row r="29" spans="3:8" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C29" s="12" t="s">
+      <c r="D30" s="20"/>
+      <c r="E30" s="20"/>
+      <c r="F30" s="14">
+        <f>F29-F28</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="3:6" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D31" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="D29" s="20"/>
-      <c r="E29" s="20"/>
-      <c r="F29" s="14">
-        <f>F28</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="3:8" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D30" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="E30" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="F30" s="2"/>
-    </row>
-    <row r="31" spans="3:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D31" s="17"/>
       <c r="E31" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="F31" s="2">
-        <f>F24</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="3:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>39</v>
+      </c>
+      <c r="F31" s="2"/>
+    </row>
+    <row r="32" spans="3:6" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D32" s="17"/>
       <c r="E32" s="7" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F32" s="2">
-        <f>F14</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="3:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+        <f>F24</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="3:6" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D33" s="17"/>
       <c r="E33" s="7" t="s">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="F33" s="2">
-        <f>F20</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="3:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
+        <f>F14</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="3:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D34" s="17"/>
       <c r="E34" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="F34" s="2"/>
-    </row>
-    <row r="35" spans="3:6" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+      <c r="F34" s="2">
+        <f>F20</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="3:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D35" s="17"/>
       <c r="E35" s="7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F35" s="2"/>
     </row>
-    <row r="36" spans="3:6" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="3:6" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D36" s="17"/>
       <c r="E36" s="7" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F36" s="2"/>
     </row>
-    <row r="37" spans="3:6" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="3:6" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D37" s="17"/>
       <c r="E37" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F37" s="2"/>
+    </row>
+    <row r="38" spans="3:6" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D38" s="17"/>
+      <c r="E38" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="F38" s="2">
+        <f>F37-F35-F34-F33-F32</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="3:6" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C39" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D39" s="20"/>
+      <c r="E39" s="20"/>
+      <c r="F39" s="14">
+        <f>F31+F36+F38</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="3:6" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D40" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="F37" s="2">
-        <f>F36-F34-F33-F32-F31</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="3:6" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C38" s="12" t="s">
+      <c r="E40" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="F40" s="2"/>
+    </row>
+    <row r="41" spans="3:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C41" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="D38" s="20"/>
-      <c r="E38" s="20"/>
-      <c r="F38" s="14">
-        <f>F30+F35+F37</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="3:6" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D39" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="E39" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="F39" s="2"/>
-    </row>
-    <row r="40" spans="3:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C40" s="12" t="s">
+      <c r="D41" s="20"/>
+      <c r="E41" s="20"/>
+      <c r="F41" s="14">
+        <f>F40</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="3:6" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D42" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="E42" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="D40" s="20"/>
-      <c r="E40" s="20"/>
-      <c r="F40" s="14">
-        <f>F39</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="3:6" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D41" s="4" t="s">
+      <c r="F42" s="2"/>
+    </row>
+    <row r="43" spans="3:6" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D43" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="E41" s="5" t="s">
+      <c r="E43" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="F41" s="2"/>
-    </row>
-    <row r="42" spans="3:6" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D42" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="E42" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="F42" s="2"/>
+      <c r="F43" s="2"/>
+    </row>
+    <row r="44" spans="3:6" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D44" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="E44" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F44" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="16">
     <mergeCell ref="D23:E23"/>
-    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="D41:E41"/>
     <mergeCell ref="D25:E25"/>
     <mergeCell ref="D27:E27"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="D30:D37"/>
-    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="D31:D38"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="D28:D29"/>
     <mergeCell ref="D6:D12"/>
     <mergeCell ref="D14:D15"/>
     <mergeCell ref="D3:F4"/>

</xml_diff>